<commit_message>
UK daily ratings for 2026-03-30
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-03-30.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-03-30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P147"/>
+  <dimension ref="A1:P219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9018,6 +9018,4304 @@
         <v>1</v>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>6</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Conquest Of Power</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>6</v>
+      </c>
+      <c r="J148" t="n">
+        <v>148</v>
+      </c>
+      <c r="K148" t="n">
+        <v>47</v>
+      </c>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P148" t="n">
+        <v>-13</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+      <c r="C149" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>6</v>
+      </c>
+      <c r="G149" t="n">
+        <v>1</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Fircombe Hall</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>8</v>
+      </c>
+      <c r="J149" t="n">
+        <v>152</v>
+      </c>
+      <c r="K149" t="n">
+        <v>51</v>
+      </c>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N149" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>1</v>
+      </c>
+      <c r="C150" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>6</v>
+      </c>
+      <c r="G150" t="n">
+        <v>2</v>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Forever Noah</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>5</v>
+      </c>
+      <c r="J150" t="n">
+        <v>155</v>
+      </c>
+      <c r="K150" t="n">
+        <v>54</v>
+      </c>
+      <c r="L150" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M150" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N150" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P150" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>6</v>
+      </c>
+      <c r="G151" t="n">
+        <v>3</v>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Instant Bond</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>5</v>
+      </c>
+      <c r="J151" t="n">
+        <v>156</v>
+      </c>
+      <c r="K151" t="n">
+        <v>55</v>
+      </c>
+      <c r="L151" t="n">
+        <v>2</v>
+      </c>
+      <c r="M151" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N151" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>6</v>
+      </c>
+      <c r="G152" t="n">
+        <v>4</v>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>No Gain</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>4</v>
+      </c>
+      <c r="J152" t="n">
+        <v>147</v>
+      </c>
+      <c r="K152" t="n">
+        <v>46</v>
+      </c>
+      <c r="L152" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="M152" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N152" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P152" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>6</v>
+      </c>
+      <c r="G153" t="n">
+        <v>5</v>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>On Key</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>4</v>
+      </c>
+      <c r="J153" t="n">
+        <v>156</v>
+      </c>
+      <c r="K153" t="n">
+        <v>55</v>
+      </c>
+      <c r="L153" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M153" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N153" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P153" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+      <c r="C154" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>6</v>
+      </c>
+      <c r="G154" t="n">
+        <v>6</v>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Spun To Gold (USA)</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>5</v>
+      </c>
+      <c r="J154" t="n">
+        <v>155</v>
+      </c>
+      <c r="K154" t="n">
+        <v>54</v>
+      </c>
+      <c r="L154" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="M154" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N154" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>6</v>
+      </c>
+      <c r="G155" t="n">
+        <v>7</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Yorkstone</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>6</v>
+      </c>
+      <c r="J155" t="n">
+        <v>151</v>
+      </c>
+      <c r="K155" t="n">
+        <v>50</v>
+      </c>
+      <c r="L155" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M155" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N155" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>6</v>
+      </c>
+      <c r="G156" t="n">
+        <v>8</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Chiedozie</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>5</v>
+      </c>
+      <c r="J156" t="n">
+        <v>147</v>
+      </c>
+      <c r="K156" t="n">
+        <v>46</v>
+      </c>
+      <c r="L156" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="M156" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N156" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P156" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>6</v>
+      </c>
+      <c r="G157" t="n">
+        <v>9</v>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Hallowed Time (IRE)</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>8</v>
+      </c>
+      <c r="J157" t="n">
+        <v>155</v>
+      </c>
+      <c r="K157" t="n">
+        <v>54</v>
+      </c>
+      <c r="L157" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="M157" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N157" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>6</v>
+      </c>
+      <c r="G158" t="n">
+        <v>10</v>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Wrist Art (IRE)</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>9</v>
+      </c>
+      <c r="J158" t="n">
+        <v>147</v>
+      </c>
+      <c r="K158" t="n">
+        <v>46</v>
+      </c>
+      <c r="L158" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M158" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N158" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>6</v>
+      </c>
+      <c r="G159" t="n">
+        <v>11</v>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Eldeyaar (IRE)</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>7</v>
+      </c>
+      <c r="J159" t="n">
+        <v>147</v>
+      </c>
+      <c r="K159" t="n">
+        <v>46</v>
+      </c>
+      <c r="L159" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="M159" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N159" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>6</v>
+      </c>
+      <c r="G160" t="n">
+        <v>12</v>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Noble Phoenix (IRE)</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>4</v>
+      </c>
+      <c r="J160" t="n">
+        <v>150</v>
+      </c>
+      <c r="K160" t="n">
+        <v>49</v>
+      </c>
+      <c r="L160" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="M160" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="N160" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>2</v>
+      </c>
+      <c r="C161" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>4</v>
+      </c>
+      <c r="G161" t="n">
+        <v>1</v>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Sovereign Spell (IRE)</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>3</v>
+      </c>
+      <c r="J161" t="n">
+        <v>129</v>
+      </c>
+      <c r="K161" t="n">
+        <v>85</v>
+      </c>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N161" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>2</v>
+      </c>
+      <c r="C162" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>4</v>
+      </c>
+      <c r="G162" t="n">
+        <v>2</v>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>The Jackal</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>3</v>
+      </c>
+      <c r="J162" t="n">
+        <v>129</v>
+      </c>
+      <c r="K162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L162" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="M162" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N162" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>2</v>
+      </c>
+      <c r="C163" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>4</v>
+      </c>
+      <c r="G163" t="n">
+        <v>3</v>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Gris De Chine</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>3</v>
+      </c>
+      <c r="J163" t="n">
+        <v>124</v>
+      </c>
+      <c r="K163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L163" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M163" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N163" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P163" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>2</v>
+      </c>
+      <c r="C164" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>4</v>
+      </c>
+      <c r="G164" t="n">
+        <v>4</v>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Royal Poetry (IRE)</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>3</v>
+      </c>
+      <c r="J164" t="n">
+        <v>124</v>
+      </c>
+      <c r="K164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L164" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="M164" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N164" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P164" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>2</v>
+      </c>
+      <c r="C165" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>4</v>
+      </c>
+      <c r="G165" t="n">
+        <v>5</v>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Lightning Hooves</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>3</v>
+      </c>
+      <c r="J165" t="n">
+        <v>129</v>
+      </c>
+      <c r="K165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" t="n">
+        <v>17.03</v>
+      </c>
+      <c r="M165" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N165" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P165" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>2</v>
+      </c>
+      <c r="C166" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>4</v>
+      </c>
+      <c r="G166" t="n">
+        <v>6</v>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Noble Gentleman (IRE)</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>3</v>
+      </c>
+      <c r="J166" t="n">
+        <v>129</v>
+      </c>
+      <c r="K166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L166" t="n">
+        <v>18.03</v>
+      </c>
+      <c r="M166" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N166" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P166" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>2</v>
+      </c>
+      <c r="C167" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>4</v>
+      </c>
+      <c r="G167" t="n">
+        <v>7</v>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Romeos Guardian</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>3</v>
+      </c>
+      <c r="J167" t="n">
+        <v>129</v>
+      </c>
+      <c r="K167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L167" t="n">
+        <v>21.03</v>
+      </c>
+      <c r="M167" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N167" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>2</v>
+      </c>
+      <c r="C168" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>4</v>
+      </c>
+      <c r="G168" t="n">
+        <v>8</v>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Cosmic Jive (IRE)</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>3</v>
+      </c>
+      <c r="J168" t="n">
+        <v>129</v>
+      </c>
+      <c r="K168" t="n">
+        <v>0</v>
+      </c>
+      <c r="L168" t="n">
+        <v>21.78</v>
+      </c>
+      <c r="M168" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N168" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>2</v>
+      </c>
+      <c r="C169" t="n">
+        <v>6.090909090909091</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>4</v>
+      </c>
+      <c r="G169" t="n">
+        <v>9</v>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Jubilee Time</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>4</v>
+      </c>
+      <c r="J169" t="n">
+        <v>142</v>
+      </c>
+      <c r="K169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L169" t="n">
+        <v>24.28</v>
+      </c>
+      <c r="M169" t="n">
+        <v>73.68000000000001</v>
+      </c>
+      <c r="N169" t="n">
+        <v>3</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P169" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>3</v>
+      </c>
+      <c r="C170" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>4</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Kings Hand</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>4</v>
+      </c>
+      <c r="J170" t="n">
+        <v>124</v>
+      </c>
+      <c r="K170" t="n">
+        <v>69</v>
+      </c>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P170" t="n">
+        <v>-13</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>3</v>
+      </c>
+      <c r="C171" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>4</v>
+      </c>
+      <c r="G171" t="n">
+        <v>1</v>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Al Durry</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>4</v>
+      </c>
+      <c r="J171" t="n">
+        <v>135</v>
+      </c>
+      <c r="K171" t="n">
+        <v>80</v>
+      </c>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N171" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>3</v>
+      </c>
+      <c r="C172" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>4</v>
+      </c>
+      <c r="G172" t="n">
+        <v>2</v>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Lordsbridge Blu</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>6</v>
+      </c>
+      <c r="J172" t="n">
+        <v>129</v>
+      </c>
+      <c r="K172" t="n">
+        <v>74</v>
+      </c>
+      <c r="L172" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M172" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N172" t="n">
+        <v>59</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P172" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>3</v>
+      </c>
+      <c r="C173" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>4</v>
+      </c>
+      <c r="G173" t="n">
+        <v>3</v>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Arcturus Flame (IRE)</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>4</v>
+      </c>
+      <c r="J173" t="n">
+        <v>132</v>
+      </c>
+      <c r="K173" t="n">
+        <v>77</v>
+      </c>
+      <c r="L173" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="M173" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N173" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P173" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>3</v>
+      </c>
+      <c r="C174" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>4</v>
+      </c>
+      <c r="G174" t="n">
+        <v>4</v>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Annexation (FR)</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>10</v>
+      </c>
+      <c r="J174" t="n">
+        <v>117</v>
+      </c>
+      <c r="K174" t="n">
+        <v>62</v>
+      </c>
+      <c r="L174" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M174" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N174" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P174" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>3</v>
+      </c>
+      <c r="C175" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>4</v>
+      </c>
+      <c r="G175" t="n">
+        <v>5</v>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Serious Look (IRE)</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>6</v>
+      </c>
+      <c r="J175" t="n">
+        <v>127</v>
+      </c>
+      <c r="K175" t="n">
+        <v>72</v>
+      </c>
+      <c r="L175" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="M175" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N175" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P175" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>3</v>
+      </c>
+      <c r="C176" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>4</v>
+      </c>
+      <c r="G176" t="n">
+        <v>6</v>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Tribal Wisdom (IRE)</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>7</v>
+      </c>
+      <c r="J176" t="n">
+        <v>134</v>
+      </c>
+      <c r="K176" t="n">
+        <v>79</v>
+      </c>
+      <c r="L176" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M176" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N176" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P176" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>3</v>
+      </c>
+      <c r="C177" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>4</v>
+      </c>
+      <c r="G177" t="n">
+        <v>7</v>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Ernies Valentine</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>7</v>
+      </c>
+      <c r="J177" t="n">
+        <v>122</v>
+      </c>
+      <c r="K177" t="n">
+        <v>67</v>
+      </c>
+      <c r="L177" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="M177" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N177" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P177" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>3</v>
+      </c>
+      <c r="C178" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>4</v>
+      </c>
+      <c r="G178" t="n">
+        <v>8</v>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Patrol (IRE)</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>4</v>
+      </c>
+      <c r="J178" t="n">
+        <v>131</v>
+      </c>
+      <c r="K178" t="n">
+        <v>76</v>
+      </c>
+      <c r="L178" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="M178" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N178" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P178" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>3</v>
+      </c>
+      <c r="C179" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>4</v>
+      </c>
+      <c r="G179" t="n">
+        <v>9</v>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Boubyan (IRE)</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>4</v>
+      </c>
+      <c r="J179" t="n">
+        <v>122</v>
+      </c>
+      <c r="K179" t="n">
+        <v>67</v>
+      </c>
+      <c r="L179" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="M179" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N179" t="n">
+        <v>37</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P179" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>3</v>
+      </c>
+      <c r="C180" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>4</v>
+      </c>
+      <c r="G180" t="n">
+        <v>10</v>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Dawn Of Liberation (IRE)</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>7</v>
+      </c>
+      <c r="J180" t="n">
+        <v>130</v>
+      </c>
+      <c r="K180" t="n">
+        <v>75</v>
+      </c>
+      <c r="L180" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="M180" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N180" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P180" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>3</v>
+      </c>
+      <c r="C181" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>4</v>
+      </c>
+      <c r="G181" t="n">
+        <v>11</v>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Criminal</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>4</v>
+      </c>
+      <c r="J181" t="n">
+        <v>131</v>
+      </c>
+      <c r="K181" t="n">
+        <v>76</v>
+      </c>
+      <c r="L181" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="M181" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N181" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P181" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>3</v>
+      </c>
+      <c r="C182" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>4</v>
+      </c>
+      <c r="G182" t="n">
+        <v>12</v>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Nedita (IRE)</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>5</v>
+      </c>
+      <c r="J182" t="n">
+        <v>124</v>
+      </c>
+      <c r="K182" t="n">
+        <v>69</v>
+      </c>
+      <c r="L182" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="M182" t="n">
+        <v>119.68</v>
+      </c>
+      <c r="N182" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P182" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>4</v>
+      </c>
+      <c r="C183" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>6</v>
+      </c>
+      <c r="G183" t="n">
+        <v>1</v>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Lux Aeterna</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>3</v>
+      </c>
+      <c r="J183" t="n">
+        <v>135</v>
+      </c>
+      <c r="K183" t="n">
+        <v>65</v>
+      </c>
+      <c r="L183" t="inlineStr"/>
+      <c r="M183" t="n">
+        <v>122.29</v>
+      </c>
+      <c r="N183" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P183" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>4</v>
+      </c>
+      <c r="C184" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>6</v>
+      </c>
+      <c r="G184" t="n">
+        <v>2</v>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Pangbourne</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>3</v>
+      </c>
+      <c r="J184" t="n">
+        <v>127</v>
+      </c>
+      <c r="K184" t="n">
+        <v>57</v>
+      </c>
+      <c r="L184" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="M184" t="n">
+        <v>122.29</v>
+      </c>
+      <c r="N184" t="n">
+        <v>40</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P184" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>4</v>
+      </c>
+      <c r="C185" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>6</v>
+      </c>
+      <c r="G185" t="n">
+        <v>3</v>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Bergamo Gold (IRE)</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>3</v>
+      </c>
+      <c r="J185" t="n">
+        <v>134</v>
+      </c>
+      <c r="K185" t="n">
+        <v>64</v>
+      </c>
+      <c r="L185" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="M185" t="n">
+        <v>122.29</v>
+      </c>
+      <c r="N185" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P185" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>4</v>
+      </c>
+      <c r="C186" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>6</v>
+      </c>
+      <c r="G186" t="n">
+        <v>4</v>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Risk Averse Rebel (IRE)</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>3</v>
+      </c>
+      <c r="J186" t="n">
+        <v>120</v>
+      </c>
+      <c r="K186" t="n">
+        <v>50</v>
+      </c>
+      <c r="L186" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="M186" t="n">
+        <v>122.29</v>
+      </c>
+      <c r="N186" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P186" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>4</v>
+      </c>
+      <c r="C187" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>6</v>
+      </c>
+      <c r="G187" t="n">
+        <v>5</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Causing Problems (IRE)</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>3</v>
+      </c>
+      <c r="J187" t="n">
+        <v>134</v>
+      </c>
+      <c r="K187" t="n">
+        <v>64</v>
+      </c>
+      <c r="L187" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="M187" t="n">
+        <v>122.29</v>
+      </c>
+      <c r="N187" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P187" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>4</v>
+      </c>
+      <c r="C188" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>6</v>
+      </c>
+      <c r="G188" t="n">
+        <v>6</v>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Frustration</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>3</v>
+      </c>
+      <c r="J188" t="n">
+        <v>130</v>
+      </c>
+      <c r="K188" t="n">
+        <v>60</v>
+      </c>
+      <c r="L188" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="M188" t="n">
+        <v>122.29</v>
+      </c>
+      <c r="N188" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P188" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>4</v>
+      </c>
+      <c r="C189" t="n">
+        <v>9.472727272727273</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>6</v>
+      </c>
+      <c r="G189" t="n">
+        <v>7</v>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Wind Summer (IRE)</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>3</v>
+      </c>
+      <c r="J189" t="n">
+        <v>133</v>
+      </c>
+      <c r="K189" t="n">
+        <v>63</v>
+      </c>
+      <c r="L189" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="M189" t="n">
+        <v>122.29</v>
+      </c>
+      <c r="N189" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P189" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>5</v>
+      </c>
+      <c r="C190" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>4</v>
+      </c>
+      <c r="G190" t="n">
+        <v>1</v>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Layla Liz (IRE)</t>
+        </is>
+      </c>
+      <c r="I190" t="n">
+        <v>4</v>
+      </c>
+      <c r="J190" t="n">
+        <v>144</v>
+      </c>
+      <c r="K190" t="n">
+        <v>87</v>
+      </c>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N190" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P190" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>5</v>
+      </c>
+      <c r="C191" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>4</v>
+      </c>
+      <c r="G191" t="n">
+        <v>2</v>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Nad Alshiba Green (IRE)</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>4</v>
+      </c>
+      <c r="J191" t="n">
+        <v>143</v>
+      </c>
+      <c r="K191" t="n">
+        <v>86</v>
+      </c>
+      <c r="L191" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M191" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N191" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P191" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>5</v>
+      </c>
+      <c r="C192" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>4</v>
+      </c>
+      <c r="G192" t="n">
+        <v>3</v>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Moes Legacy</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>5</v>
+      </c>
+      <c r="J192" t="n">
+        <v>132</v>
+      </c>
+      <c r="K192" t="n">
+        <v>75</v>
+      </c>
+      <c r="L192" t="n">
+        <v>1</v>
+      </c>
+      <c r="M192" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N192" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P192" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>5</v>
+      </c>
+      <c r="C193" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>4</v>
+      </c>
+      <c r="G193" t="n">
+        <v>4</v>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Saucy Jane</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>3</v>
+      </c>
+      <c r="J193" t="n">
+        <v>125</v>
+      </c>
+      <c r="K193" t="n">
+        <v>80</v>
+      </c>
+      <c r="L193" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M193" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N193" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P193" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>5</v>
+      </c>
+      <c r="C194" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>4</v>
+      </c>
+      <c r="G194" t="n">
+        <v>5</v>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Angel Numbers (IRE)</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>3</v>
+      </c>
+      <c r="J194" t="n">
+        <v>121</v>
+      </c>
+      <c r="K194" t="n">
+        <v>76</v>
+      </c>
+      <c r="L194" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M194" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N194" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P194" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>5</v>
+      </c>
+      <c r="C195" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>4</v>
+      </c>
+      <c r="G195" t="n">
+        <v>6</v>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Ophelia Grace (IRE)</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>3</v>
+      </c>
+      <c r="J195" t="n">
+        <v>128</v>
+      </c>
+      <c r="K195" t="n">
+        <v>83</v>
+      </c>
+      <c r="L195" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M195" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N195" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P195" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>5</v>
+      </c>
+      <c r="C196" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>4</v>
+      </c>
+      <c r="G196" t="n">
+        <v>7</v>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Sams Hope</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>6</v>
+      </c>
+      <c r="J196" t="n">
+        <v>134</v>
+      </c>
+      <c r="K196" t="n">
+        <v>77</v>
+      </c>
+      <c r="L196" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="M196" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N196" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P196" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>5</v>
+      </c>
+      <c r="C197" t="n">
+        <v>5.095454545454546</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>4</v>
+      </c>
+      <c r="G197" t="n">
+        <v>8</v>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Nifty (IRE)</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>3</v>
+      </c>
+      <c r="J197" t="n">
+        <v>118</v>
+      </c>
+      <c r="K197" t="n">
+        <v>73</v>
+      </c>
+      <c r="L197" t="n">
+        <v>8</v>
+      </c>
+      <c r="M197" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="N197" t="n">
+        <v>34</v>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P197" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>6</v>
+      </c>
+      <c r="C198" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>6</v>
+      </c>
+      <c r="G198" t="n">
+        <v>1</v>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Bossy Parker (IRE)</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>6</v>
+      </c>
+      <c r="J198" t="n">
+        <v>135</v>
+      </c>
+      <c r="K198" t="n">
+        <v>48</v>
+      </c>
+      <c r="L198" t="inlineStr"/>
+      <c r="M198" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N198" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P198" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>6</v>
+      </c>
+      <c r="C199" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>6</v>
+      </c>
+      <c r="G199" t="n">
+        <v>2</v>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Alpine Sierra (IRE)</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>8</v>
+      </c>
+      <c r="J199" t="n">
+        <v>135</v>
+      </c>
+      <c r="K199" t="n">
+        <v>50</v>
+      </c>
+      <c r="L199" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M199" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N199" t="n">
+        <v>64</v>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P199" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>6</v>
+      </c>
+      <c r="C200" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>6</v>
+      </c>
+      <c r="G200" t="n">
+        <v>3</v>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Nutcracker</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>4</v>
+      </c>
+      <c r="J200" t="n">
+        <v>135</v>
+      </c>
+      <c r="K200" t="n">
+        <v>45</v>
+      </c>
+      <c r="L200" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M200" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N200" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P200" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>6</v>
+      </c>
+      <c r="C201" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>6</v>
+      </c>
+      <c r="G201" t="n">
+        <v>4</v>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Pebble Dash (IRE)</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>4</v>
+      </c>
+      <c r="J201" t="n">
+        <v>135</v>
+      </c>
+      <c r="K201" t="n">
+        <v>49</v>
+      </c>
+      <c r="L201" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="M201" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N201" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P201" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>6</v>
+      </c>
+      <c r="C202" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>6</v>
+      </c>
+      <c r="G202" t="n">
+        <v>5</v>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Star Of Atlantis (IRE)</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>5</v>
+      </c>
+      <c r="J202" t="n">
+        <v>135</v>
+      </c>
+      <c r="K202" t="n">
+        <v>49</v>
+      </c>
+      <c r="L202" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="M202" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N202" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P202" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>6</v>
+      </c>
+      <c r="C203" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>6</v>
+      </c>
+      <c r="G203" t="n">
+        <v>6</v>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Spinning Dancer (IRE)</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>4</v>
+      </c>
+      <c r="J203" t="n">
+        <v>135</v>
+      </c>
+      <c r="K203" t="n">
+        <v>45</v>
+      </c>
+      <c r="L203" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="M203" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N203" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P203" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>6</v>
+      </c>
+      <c r="C204" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>6</v>
+      </c>
+      <c r="G204" t="n">
+        <v>7</v>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Man Is King (IRE)</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>7</v>
+      </c>
+      <c r="J204" t="n">
+        <v>135</v>
+      </c>
+      <c r="K204" t="n">
+        <v>49</v>
+      </c>
+      <c r="L204" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="M204" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N204" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P204" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>6</v>
+      </c>
+      <c r="C205" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>6</v>
+      </c>
+      <c r="G205" t="n">
+        <v>8</v>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Boomtown Lad (IRE)</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>4</v>
+      </c>
+      <c r="J205" t="n">
+        <v>135</v>
+      </c>
+      <c r="K205" t="n">
+        <v>35</v>
+      </c>
+      <c r="L205" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="M205" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N205" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P205" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>6</v>
+      </c>
+      <c r="C206" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>6</v>
+      </c>
+      <c r="G206" t="n">
+        <v>9</v>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Galette</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>4</v>
+      </c>
+      <c r="J206" t="n">
+        <v>135</v>
+      </c>
+      <c r="K206" t="n">
+        <v>40</v>
+      </c>
+      <c r="L206" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="M206" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N206" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P206" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>6</v>
+      </c>
+      <c r="C207" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>6</v>
+      </c>
+      <c r="G207" t="n">
+        <v>10</v>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Lhebayeb (GER)</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>8</v>
+      </c>
+      <c r="J207" t="n">
+        <v>135</v>
+      </c>
+      <c r="K207" t="n">
+        <v>50</v>
+      </c>
+      <c r="L207" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="M207" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N207" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P207" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>6</v>
+      </c>
+      <c r="C208" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>6</v>
+      </c>
+      <c r="G208" t="n">
+        <v>11</v>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Wingstar (IRE)</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>4</v>
+      </c>
+      <c r="J208" t="n">
+        <v>135</v>
+      </c>
+      <c r="K208" t="n">
+        <v>46</v>
+      </c>
+      <c r="L208" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="M208" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="N208" t="n">
+        <v>37</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P208" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>7</v>
+      </c>
+      <c r="C209" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>6</v>
+      </c>
+      <c r="G209" t="n">
+        <v>1</v>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Captain Pickles (IRE)</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>4</v>
+      </c>
+      <c r="J209" t="n">
+        <v>131</v>
+      </c>
+      <c r="K209" t="n">
+        <v>51</v>
+      </c>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N209" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P209" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>7</v>
+      </c>
+      <c r="C210" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>6</v>
+      </c>
+      <c r="G210" t="n">
+        <v>2</v>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Brinton</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>5</v>
+      </c>
+      <c r="J210" t="n">
+        <v>134</v>
+      </c>
+      <c r="K210" t="n">
+        <v>54</v>
+      </c>
+      <c r="L210" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M210" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N210" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P210" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>7</v>
+      </c>
+      <c r="C211" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>6</v>
+      </c>
+      <c r="G211" t="n">
+        <v>3</v>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Arlecchinos Rex</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>4</v>
+      </c>
+      <c r="J211" t="n">
+        <v>129</v>
+      </c>
+      <c r="K211" t="n">
+        <v>49</v>
+      </c>
+      <c r="L211" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M211" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N211" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P211" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>7</v>
+      </c>
+      <c r="C212" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>6</v>
+      </c>
+      <c r="G212" t="n">
+        <v>4</v>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Princess Vivi</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>4</v>
+      </c>
+      <c r="J212" t="n">
+        <v>126</v>
+      </c>
+      <c r="K212" t="n">
+        <v>46</v>
+      </c>
+      <c r="L212" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M212" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N212" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P212" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>7</v>
+      </c>
+      <c r="C213" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>6</v>
+      </c>
+      <c r="G213" t="n">
+        <v>5</v>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Sceptic (IRE)</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>6</v>
+      </c>
+      <c r="J213" t="n">
+        <v>135</v>
+      </c>
+      <c r="K213" t="n">
+        <v>55</v>
+      </c>
+      <c r="L213" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M213" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N213" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P213" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>7</v>
+      </c>
+      <c r="C214" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F214" t="n">
+        <v>6</v>
+      </c>
+      <c r="G214" t="n">
+        <v>6</v>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>First Encounter</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>5</v>
+      </c>
+      <c r="J214" t="n">
+        <v>131</v>
+      </c>
+      <c r="K214" t="n">
+        <v>51</v>
+      </c>
+      <c r="L214" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="M214" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N214" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P214" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>7</v>
+      </c>
+      <c r="C215" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>6</v>
+      </c>
+      <c r="G215" t="n">
+        <v>7</v>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Mooretown Lad (IRE)</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>6</v>
+      </c>
+      <c r="J215" t="n">
+        <v>132</v>
+      </c>
+      <c r="K215" t="n">
+        <v>52</v>
+      </c>
+      <c r="L215" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M215" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N215" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P215" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>7</v>
+      </c>
+      <c r="C216" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>6</v>
+      </c>
+      <c r="G216" t="n">
+        <v>8</v>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Wyvern</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>7</v>
+      </c>
+      <c r="J216" t="n">
+        <v>134</v>
+      </c>
+      <c r="K216" t="n">
+        <v>54</v>
+      </c>
+      <c r="L216" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M216" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N216" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P216" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>7</v>
+      </c>
+      <c r="C217" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>6</v>
+      </c>
+      <c r="G217" t="n">
+        <v>9</v>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Like Magic (GER)</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>5</v>
+      </c>
+      <c r="J217" t="n">
+        <v>132</v>
+      </c>
+      <c r="K217" t="n">
+        <v>52</v>
+      </c>
+      <c r="L217" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="M217" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N217" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P217" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>7</v>
+      </c>
+      <c r="C218" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>6</v>
+      </c>
+      <c r="G218" t="n">
+        <v>10</v>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Take The A Train</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>4</v>
+      </c>
+      <c r="J218" t="n">
+        <v>131</v>
+      </c>
+      <c r="K218" t="n">
+        <v>51</v>
+      </c>
+      <c r="L218" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="M218" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N218" t="n">
+        <v>40</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P218" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>WOLVERHAMPTON</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>7</v>
+      </c>
+      <c r="C219" t="n">
+        <v>8.645454545454545</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>6</v>
+      </c>
+      <c r="G219" t="n">
+        <v>11</v>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>Morning Suit (IRE)</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>5</v>
+      </c>
+      <c r="J219" t="n">
+        <v>126</v>
+      </c>
+      <c r="K219" t="n">
+        <v>46</v>
+      </c>
+      <c r="L219" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="M219" t="n">
+        <v>109.83</v>
+      </c>
+      <c r="N219" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P219" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>